<commit_message>
fix(phase15d): pharma and cosmetic page corrections, intro fixes, and linter hardening
</commit_message>
<xml_diff>
--- a/phase15/spec-confirmation.xlsx
+++ b/phase15/spec-confirmation.xlsx
@@ -730,13 +730,13 @@
       <c r="G6" s="5" t="n"/>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>10 Claims</t>
+          <t>12 Claims</t>
         </is>
       </c>
       <c r="I6" s="5" t="n"/>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>68 Items</t>
+          <t>70 Items</t>
         </is>
       </c>
       <c r="K6" s="5" t="n"/>
@@ -1182,7 +1182,7 @@
       </c>
       <c r="E27" s="15" t="inlineStr">
         <is>
-          <t>Regular Supply</t>
+          <t>Available on Enquiry</t>
         </is>
       </c>
       <c r="F27" s="15" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Regular Supply</t>
+          <t>Available on Enquiry</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>10 additional claims in 'Claims to confirm' sheet (Grand Total: 68 items)</t>
+          <t>12 additional claims in 'Claims to confirm' sheet (Grand Total: 70 items)</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1558,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="20" t="inlineStr">
         <is>
-          <t>NAGDEV PRODUCTS — PALE PRESSED GRADE (PPG) CASTOR OIL (NDEVOLEO™ PPG) | Category: Castor Oils | Status: Regular Supply</t>
+          <t>NAGDEV PRODUCTS — PALE PRESSED GRADE (PPG) CASTOR OIL (NDEVOLEO™ PPG) | Category: Castor Oils | Status: Available on Enquiry</t>
         </is>
       </c>
     </row>
@@ -2089,7 +2089,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="20" t="inlineStr">
         <is>
-          <t>NAGDEV PRODUCTS — COLD PRESSED CASTOR OIL (NDEVOLEO™ CP) | Category: Specialty Castor Oils | Status: Regular Supply</t>
+          <t>NAGDEV PRODUCTS — COLD PRESSED CASTOR OIL (NDEVOLEO™ CP) | Category: Specialty Castor Oils | Status: Available on Enquiry</t>
         </is>
       </c>
     </row>
@@ -3198,12 +3198,12 @@
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="23" t="inlineStr">
         <is>
-          <t>Heavy Metals</t>
+          <t>Elemental impurities (as required by the current USP–NF)</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>ppm</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C8" s="16" t="inlineStr">
@@ -4424,7 +4424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4817,13 +4817,79 @@
       </c>
       <c r="G13" s="24" t="inlineStr"/>
     </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t>Packaging: Pharma &amp; Cosmetic Bulk</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Pharma/cosmetic bulk in flexitank/ISO tank — offered?</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>spec-confirmation.xlsx, products/castor-oil-*.html, cosmetic-grade-castor-oil.html</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>Awaiting Owner Confirmation</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="F14" s="16" t="inlineStr">
+        <is>
+          <t>Owner confirmation required before offering flexitanks or ISO tanks for pharma and cosmetic castor oil grades.</t>
+        </is>
+      </c>
+      <c r="G14" s="24" t="inlineStr"/>
+    </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="25" t="inlineStr">
+        <is>
+          <t>Ph. Eur. Castor Oil Monograph Scope</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Which Ph. Eur. monograph(s) can be supplied — virgin, refined, or both?</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>spec-confirmation.xlsx, products/castor-oil-ph-eur.html, downloads/tds/castor-oil-ph-eur.pdf</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Awaiting Owner Confirmation</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>The Ph. Eur. has separate monographs for virgin castor oil and refined castor oil. Specify which monograph(s) Nagdev Products supplies.</t>
+        </is>
+      </c>
+      <c r="G15" s="24" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Keep,Change,Remove"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>